<commit_message>
them modifi option 2
</commit_message>
<xml_diff>
--- a/logistics/scenario_output/monthly_logistics_cost.xlsx
+++ b/logistics/scenario_output/monthly_logistics_cost.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly_Logistics_Cost" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly_Detail" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary_by_Market" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario_Cost_Breakdown" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Monthly_Logistics_Cost" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Weekly_Detail" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary_by_Market" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Scenario_Cost_Breakdown" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -780,10 +780,10 @@
         <v>9000</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>4928.44</v>
+        <v>4928.18</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>19128.44</v>
+        <v>19128.18</v>
       </c>
     </row>
     <row r="8">
@@ -1599,10 +1599,10 @@
         <v>6000</v>
       </c>
       <c r="J28" s="4" t="n">
-        <v>1790.69</v>
+        <v>1790.56</v>
       </c>
       <c r="K28" s="4" t="n">
-        <v>7790.69</v>
+        <v>7790.56</v>
       </c>
     </row>
     <row r="29">
@@ -1635,10 +1635,10 @@
         <v>96000</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>62430.44</v>
+        <v>62430.05</v>
       </c>
       <c r="L29" s="7" t="n">
-        <v>168830.44</v>
+        <v>168830.05</v>
       </c>
     </row>
   </sheetData>
@@ -2552,7 +2552,7 @@
         <v>1</v>
       </c>
       <c r="H20" s="9" t="n">
-        <v>10.266875</v>
+        <v>10.265625</v>
       </c>
       <c r="I20" s="4" t="n">
         <v>0</v>
@@ -2561,10 +2561,10 @@
         <v>3000</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>2053.38</v>
+        <v>2053.12</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>5053.38</v>
+        <v>5053.12</v>
       </c>
     </row>
     <row r="21">
@@ -6380,7 +6380,7 @@
         <v>1</v>
       </c>
       <c r="H107" s="9" t="n">
-        <v>4.472188</v>
+        <v>4.471563</v>
       </c>
       <c r="I107" s="4" t="n">
         <v>0</v>
@@ -6389,10 +6389,10 @@
         <v>3000</v>
       </c>
       <c r="K107" s="4" t="n">
-        <v>894.4400000000001</v>
+        <v>894.3099999999999</v>
       </c>
       <c r="L107" s="4" t="n">
-        <v>3894.44</v>
+        <v>3894.31</v>
       </c>
     </row>
     <row r="108">
@@ -6505,7 +6505,7 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6633,7 +6633,7 @@
         <v>32</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>153.201563</v>
+        <v>153.199688</v>
       </c>
       <c r="F4" s="4" t="n">
         <v>10400</v>
@@ -6642,10 +6642,10 @@
         <v>96000</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>30640.3</v>
+        <v>30639.91</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>137040.3</v>
+        <v>137039.91</v>
       </c>
     </row>
   </sheetData>
@@ -6700,7 +6700,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>137040.3</v>
+        <v>137039.91</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -6745,7 +6745,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>168830.44</v>
+        <v>168830.05</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -6831,7 +6831,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>168830.44</v>
+        <v>168830.05</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -6861,7 +6861,7 @@
         </is>
       </c>
       <c r="B16" s="12" t="n">
-        <v>238870.44</v>
+        <v>238870.05</v>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>

</xml_diff>